<commit_message>
Fix result notifications report
</commit_message>
<xml_diff>
--- a/api/templates/result_notifications/uk.xlsx
+++ b/api/templates/result_notifications/uk.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="33">
   <si>
     <t xml:space="preserve">SMS-повідомлення</t>
   </si>
@@ -50,70 +50,70 @@
     <t xml:space="preserve">Мобільний телефон</t>
   </si>
   <si>
+    <t xml:space="preserve">повідомлення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Надіслано</t>
+  </si>
+  <si>
+    <t xml:space="preserve">пристрій</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ID пацієнта</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ідентифікатор зразка</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Дата тестування</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Текст результату</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;notification&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;recipient&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;mobilePhone&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;message&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;sentOn&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;device&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;patientId&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;sampleId&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;endedOn&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;resultText&gt;</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сповіщення електронною поштою</t>
+  </si>
+  <si>
     <t xml:space="preserve">Електронна пошта</t>
   </si>
   <si>
-    <t xml:space="preserve">повідомлення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Надіслано</t>
-  </si>
-  <si>
-    <t xml:space="preserve">пристрій</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ID пацієнта</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ідентифікатор зразка</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Дата тестування</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Текст результату</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;notification&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;recipient&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;mobilePhone&gt;</t>
+    <t xml:space="preserve">Тема</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Тіло</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;email&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;message&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;sentOn&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;device&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;patientId&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;sampleId&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;endedOn&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;resultText&gt;</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сповіщення електронною поштою</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Тема</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Тіло</t>
   </si>
   <si>
     <t xml:space="preserve">&lt;subject&gt;</t>
@@ -256,8 +256,12 @@
       <protection locked="true" hidden="false"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -293,16 +297,8 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -387,134 +383,124 @@
   <dimension ref="A1:K12"/>
   <sheetFormatPr defaultColWidth="11.30078125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="27.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="30.1"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="15.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="43.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="17.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="53.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="27.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="19.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15.3"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="15.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="43.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="16.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="17.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="15.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="53.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="9.34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
+      <c r="C1" s="2"/>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+      <c r="A3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="3"/>
+      <c r="C3" s="4"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+      <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+      <c r="A5" s="3" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4"/>
-    </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A6" s="5"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="8" s="6" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+    <row r="8" s="7" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="G8" s="5" t="s">
+      <c r="G8" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="H8" s="5" t="s">
+      <c r="H8" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="I8" s="5" t="s">
+      <c r="I8" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="J8" s="5" t="s">
+      <c r="J8" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="K8" s="5" t="s">
+      <c r="K8" s="0"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
+      <c r="B9" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="C9" s="8" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="7" t="s">
+      <c r="D9" s="8" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="7" t="s">
+      <c r="E9" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="7" t="s">
+      <c r="F9" s="8" t="s">
         <v>21</v>
       </c>
-      <c r="F9" s="8" t="s">
+      <c r="G9" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="G9" s="7" t="s">
+      <c r="H9" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="I9" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="J9" s="8" t="s">
         <v>25</v>
-      </c>
-      <c r="J9" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="K9" s="7" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="C3:D3"/>
-  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -533,143 +519,132 @@
   <dimension ref="A1:L12"/>
   <sheetFormatPr defaultColWidth="11.30078125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="27.5"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="19.3"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="0" width="30.1"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="33.8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="15.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="53.1"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="16.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="17.6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="15.2"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="53.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="24.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="27.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="30.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="33.8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="15.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="53.1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="17.6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="15.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="1" width="53.2"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="9.34"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="21" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="4"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="5"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" s="7" customFormat="true" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="4"/>
-    </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" s="6" customFormat="true" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" s="5" t="s">
+      <c r="E8" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F8" s="5" t="s">
+      <c r="F8" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="G8" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H8" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="J8" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="K8" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="L8" s="0"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C9" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="G8" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="H8" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="I8" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="J8" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="K8" s="5" t="s">
-        <v>15</v>
-      </c>
-      <c r="L8" s="5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B9" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" s="7" t="s">
+      <c r="D9" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F9" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="7" t="s">
-        <v>31</v>
-      </c>
-      <c r="F9" s="7" t="s">
-        <v>32</v>
-      </c>
       <c r="G9" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="H9" s="8" t="s">
         <v>22</v>
       </c>
-      <c r="H9" s="7" t="s">
+      <c r="I9" s="8" t="s">
         <v>23</v>
       </c>
-      <c r="I9" s="7" t="s">
+      <c r="J9" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="J9" s="7" t="s">
+      <c r="K9" s="8" t="s">
         <v>25</v>
-      </c>
-      <c r="K9" s="8" t="s">
-        <v>26</v>
-      </c>
-      <c r="L9" s="7" t="s">
-        <v>27</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="10"/>
       <c r="C12" s="10"/>
       <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="C3:D3"/>
-  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>